<commit_message>
chore: recover and synchronize office workstation changes
</commit_message>
<xml_diff>
--- a/public/as-made/files/AS-MADE_siemens-12.xlsx
+++ b/public/as-made/files/AS-MADE_siemens-12.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="רשימות" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'הוראות מילוי · تعليمات'!$A$1:$B$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'הוראות מילוי · تعليمات'!$A$1:$B$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'טופס AS-MADE'!$10:$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -77,6 +77,10 @@
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <i val="1"/>
       <color rgb="009CA3AF"/>
       <sz val="10"/>
@@ -105,10 +109,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="7">
@@ -176,16 +176,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -220,14 +220,14 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -235,8 +235,8 @@
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -701,211 +701,197 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="15" customHeight="1">
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>•  בבקרי תריסים: "זמן נסיעה מלא" — כמה שניות לוקח לתריס לרדת מפתוח לגמרי לסגור לגמרי. מדוד/י בפועל עם סטופר. בלי הזמן הזה אי אפשר לתכנת מיקום באחוזים.</t>
+          <t>•  "נבדק בשטח" — סמן/י "כן" רק אחרי שהפעלת את המעגל וראית שהוא עובד.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>•  "נבדק בשטח" — סמן/י "כן" רק אחרי שהפעלת את המעגל וראית שהוא עובד.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="B17" s="6" t="inlineStr">
-        <is>
           <t>•  ערוץ שאינו בשימוש — השאר/י ריק. אל תמחק/י את השורה.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="21" customHeight="1">
-      <c r="B18" s="5" t="inlineStr">
+    <row r="17" ht="21" customHeight="1">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>מה לא ממלאים</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="28" customHeight="1">
-      <c r="B19" s="6" t="inlineStr">
+    <row r="18" ht="28" customHeight="1">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>•  כל תא אפור שרשום בו "ימולא ע"י I FEEL" — נעול. הכתובת הפיזית, כתובות הקבוצה ושמות האובייקטים ב-ETS נקבעים אצלנו בשלב התכנות.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="21" customHeight="1">
-      <c r="B20" s="5" t="inlineStr">
+    <row r="19" ht="21" customHeight="1">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>שליחה</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="28" customHeight="1">
+    <row r="20" ht="28" customHeight="1">
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>•  מלא/י באתר i-feel.co.il ולחץ/י "שליחה" — הטופס מגיע ישירות למנהל הפרויקט, או שמור/י את הקובץ ושלח/י אותו במייל.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>•  מלא/י באתר i-feel.co.il ולחץ/י "שליחה" — הטופס מגיע ישירות למנהל הפרויקט, או שמור/י את הקובץ ושלח/י אותו במייל.</t>
+          <t>•  מומלץ לצרף גם צילום של הלוח הפתוח ושל סימון הכבלים.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>•  מומלץ לצרף גם צילום של הלוח הפתוח ושל סימון הכבלים.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1">
-      <c r="B23" s="6" t="inlineStr">
-        <is>
           <t>•  שאלות: I FEEL · 03-508-9553 · i-feel.co.il</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="26" customHeight="1">
-      <c r="B26" s="3" t="inlineStr">
+    <row r="25" ht="26" customHeight="1">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>كيفية تعبئة النموذج — تعليمات للكهربائي</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="B27" s="4" t="inlineStr">
+    <row r="26" ht="30" customHeight="1">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>هذا النموذج هو مخطط AS-MADE للوحة الكهرباء. بناءً عليه نقوم في I FEEL ببرمجة وحدات التحكم في ETS6. ما لا يُكتب هنا — لن تتم برمجته.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="21" customHeight="1">
-      <c r="B28" s="5" t="inlineStr">
+    <row r="27" ht="21" customHeight="1">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>قبل البدء</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>•  تأكّد من أن اللوحة موصولة فعلياً وأن ترقيم الكابلات مطابق لما هو مكتوب في النموذج.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>•  تأكّد من أن اللوحة موصولة فعلياً وأن ترقيم الكابلات مطابق لما هو مكتوب في النموذج.</t>
+          <t>•  عبّئ تفاصيل المشروع في أعلى النموذج: اسم المشروع، عنوان الموقع، رقم اللوحة، اسمك، رقم هاتفك وبريدك الإلكتروني.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>•  عبّئ تفاصيل المشروع في أعلى النموذج: اسم المشروع، عنوان الموقع، رقم اللوحة، اسمك، رقم هاتفك وبريدك الإلكتروني.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="B31" s="6" t="inlineStr">
-        <is>
           <t>•  إذا كانت اللوحة تحتوي على عدة وحدات من النوع نفسه — النموذج مقسّم مسبقاً إلى كتل: وحدة P1، وحدة P2 وهكذا. الوحدة غير الموجودة — اترك كتلتها فارغة.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="21" customHeight="1">
-      <c r="B32" s="5" t="inlineStr">
+    <row r="31" ht="21" customHeight="1">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>التعبئة سطراً سطراً</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1">
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>•  كل سطر = قناة واحدة في وحدة التحكم. ترتيب القنوات في النموذج مطابق لترتيب المشابك.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>•  كل سطر = قناة واحدة في وحدة التحكم. ترتيب القنوات في النموذج مطابق لترتيب المشابك.</t>
+          <t>•  "الغرفة / المنطقة" — اسم الغرفة كما يسميها الزبون: صالون، مطبخ، غرفة نوم، شرفة.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>•  "الغرفة / المنطقة" — اسم الغرفة كما يسميها الزبون: صالون، مطبخ، غرفة نوم، شرفة.</t>
+          <t>•  "وصف الدائرة / الحمل" — ما هو الموصول فعلياً: سبوتات المطبخ، ثريا غرفة الطعام، إنارة الحديقة.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>•  "وصف الدائرة / الحمل" — ما هو الموصول فعلياً: سبوتات المطبخ، ثريا غرفة الطعام، إنارة الحديقة.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="28" customHeight="1">
+          <t>•  "نوع الحمل" و"الوظيفة المطلوبة" — اختر من القائمة المنسدلة فقط. لا تكتب نصاً حراً.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1">
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>•  "نوع الحمل" و"الوظيفة المطلوبة" — اختر من القائمة المنسدلة فقط. لا تكتب نصاً حراً.</t>
+          <t>•  "القدرة / الكمية" — تيار القاطع (مثلاً 10A) أو القدرة بالواط.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>•  "القدرة / الكمية" — تيار القاطع (مثلاً 10A) أو القدرة بالواط.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="41" customHeight="1">
+          <t>•  "تم الفحص في الموقع" — ضع "نعم" فقط بعد تشغيل الدائرة والتأكد من عملها.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="15" customHeight="1">
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>•  في وحدات الستائر: "زمن الحركة الكامل" — كم ثانية تحتاج الستارة للنزول من الفتح الكامل حتى الإغلاق الكامل. قِس بساعة إيقاف. بدون هذا الزمن لا يمكن برمجة الموضع بالنسبة المئوية.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="15" customHeight="1">
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>•  "تم الفحص في الموقع" — ضع "نعم" فقط بعد تشغيل الدائرة والتأكد من عملها.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="15" customHeight="1">
+          <t>•  القناة غير المستخدمة — اتركها فارغة. لا تحذف السطر.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="21" customHeight="1">
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>ما لا يجب تعبئته</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="28" customHeight="1">
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>•  القناة غير المستخدمة — اتركها فارغة. لا تحذف السطر.</t>
+          <t>•  كل خانة رمادية مكتوب فيها "ימולא ע"י I FEEL" — مقفلة. العنوان الفيزيائي وعناوين المجموعات وأسماء الكائنات في ETS تُحدَّد لدينا في مرحلة البرمجة.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="21" customHeight="1">
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>ما لا يجب تعبئته</t>
+          <t>الإرسال</t>
         </is>
       </c>
     </row>
     <row r="42" ht="28" customHeight="1">
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>•  كل خانة رمادية مكتوب فيها "ימולא ע"י I FEEL" — مقفلة. العنوان الفيزيائي وعناوين المجموعات وأسماء الكائنات في ETS تُحدَّد لدينا في مرحلة البرمجة.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="21" customHeight="1">
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>الإرسال</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="28" customHeight="1">
+          <t>•  عبّئ النموذج في موقع i-feel.co.il واضغط "إرسال" — يصل مباشرة إلى مدير المشروع، أو احفظ الملف وأرسله بالبريد الإلكتروني.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15" customHeight="1">
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>•  يُفضّل إرفاق صورة للوحة مفتوحة ولترقيم الكابلات.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15" customHeight="1">
       <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>•  عبّئ النموذج في موقع i-feel.co.il واضغط "إرسال" — يصل مباشرة إلى مدير المشروع، أو احفظ الملف وأرسله بالبريد الإلكتروني.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="15" customHeight="1">
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>•  يُفضّل إرفاق صورة للوحة مفتوحة ولترقيم الكابلات.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="15" customHeight="1">
-      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>•  للاستفسار: I FEEL · 03-508-9553 · i-feel.co.il</t>
         </is>

</xml_diff>